<commit_message>
V0.3: automatic merchant categorization + UPI threshold rule + needs-review list
</commit_message>
<xml_diff>
--- a/data/sample_statement.xlsx
+++ b/data/sample_statement.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pritish\Documents\CreditCardAnalyserProject\V0.1\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pritish\Documents\CreditCardAnalyserProject\v0.3\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B89C2FF-B128-4B33-8B30-C9D877F1C045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F62CF6-DD64-4BFA-8F02-7A6E57708F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{0CE1568C-E725-42CE-92BA-E11B93FDA9F5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" xr2:uid="{0CE1568C-E725-42CE-92BA-E11B93FDA9F5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>Date</t>
   </si>
@@ -73,6 +73,15 @@
   </si>
   <si>
     <t>Tax</t>
+  </si>
+  <si>
+    <t>Local Kirana Store</t>
+  </si>
+  <si>
+    <t>UPI-9876543210-Ramesh Kirana</t>
+  </si>
+  <si>
+    <t>UPI-9988776655-Chai Wala</t>
   </si>
 </sst>
 </file>
@@ -108,9 +117,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -425,8 +440,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB3106AD-31E9-429E-9540-F251FD60F3D8}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.5703125" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -512,6 +531,48 @@
         <v>12</v>
       </c>
     </row>
+    <row r="7" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>46034</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="3">
+        <v>1200</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>46035</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="3">
+        <v>450</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>46036</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3">
+        <v>50</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>